<commit_message>
Fix: fix refreshing crafting list bug and add interaction text data to chest and crafting table
</commit_message>
<xml_diff>
--- a/DataSources/CraftingRecipes.xlsx
+++ b/DataSources/CraftingRecipes.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\DataSources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\Unreal Projects\AWeek\DataSources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35E72959-C083-407D-9A09-513556D85ABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2FD2E71-0525-4FB7-AE5A-CFF811C92D13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="510" yWindow="1980" windowWidth="14700" windowHeight="13080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6540" yWindow="3000" windowWidth="21315" windowHeight="13080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t>CraftedItem</t>
   </si>
@@ -93,15 +93,6 @@
     <t>RefinedMetalBundle:1, BoxOfNails:1</t>
   </si>
   <si>
-    <t>RevolverHandgun:1</t>
-  </si>
-  <si>
-    <t>IronPipes:1, RefinedMetalBundle:2, DuctTape:1</t>
-  </si>
-  <si>
-    <t>HuntingRifle:1</t>
-  </si>
-  <si>
     <t>WoodenPlank:4, IronPipes:2, RefinedMetalBundle:2</t>
   </si>
   <si>
@@ -117,15 +108,9 @@
     <t>SmallFirstAidKit:3, RefinedMetalBundle:1</t>
   </si>
   <si>
-    <t>AssaultRifle_01:1</t>
-  </si>
-  <si>
     <t>RefinedMetalBundle:4, IronPipes:2, ScrapElectronics:1</t>
   </si>
   <si>
-    <t>TacticalCarbine:1</t>
-  </si>
-  <si>
     <t>RefinedMetalBundle:3, IronPipes:2, ScrapElectronics:2, DuctTape:2</t>
   </si>
   <si>
@@ -150,24 +135,12 @@
     <t>RefinedMetalBundle</t>
   </si>
   <si>
-    <t>RevolverHandgun</t>
-  </si>
-  <si>
-    <t>HuntingRifle</t>
-  </si>
-  <si>
     <t>CarBattery</t>
   </si>
   <si>
     <t>AdvancedMedicalCrate</t>
   </si>
   <si>
-    <t>AssaultRifle_01</t>
-  </si>
-  <si>
-    <t>TacticalCarbine</t>
-  </si>
-  <si>
     <t>Rope</t>
   </si>
   <si>
@@ -201,13 +174,33 @@
     <t>WoodenPlank:3, IronPipes:1, BoxOfNails:2</t>
   </si>
   <si>
-    <t>HeavyRifle_AK</t>
-  </si>
-  <si>
-    <t>HeavyRifle_AK:1</t>
-  </si>
-  <si>
     <t>RefinedMetalBundle:4, WoodLog:1, ScrapElectronics:1</t>
+  </si>
+  <si>
+    <t>Rifle_4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Rifle_1</t>
+  </si>
+  <si>
+    <t>Rifle_1:1</t>
+  </si>
+  <si>
+    <t>Rifle_2</t>
+  </si>
+  <si>
+    <t>Rifle_2:1</t>
+  </si>
+  <si>
+    <t>Rifle_3</t>
+  </si>
+  <si>
+    <t>Rifle_3:1</t>
+  </si>
+  <si>
+    <t>Rifle_4:1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -532,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.125" bestFit="1" customWidth="1"/>
@@ -544,7 +537,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -572,7 +565,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
@@ -586,7 +579,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B4" t="s">
         <v>10</v>
@@ -600,7 +593,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B5" t="s">
         <v>12</v>
@@ -614,7 +607,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B6" t="s">
         <v>14</v>
@@ -628,7 +621,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
         <v>16</v>
@@ -642,7 +635,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
         <v>18</v>
@@ -670,13 +663,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="B10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" t="s">
         <v>22</v>
-      </c>
-      <c r="C10" t="s">
-        <v>23</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -684,13 +677,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" t="s">
         <v>24</v>
-      </c>
-      <c r="C11" t="s">
-        <v>25</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -698,13 +691,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" t="s">
         <v>26</v>
-      </c>
-      <c r="C12" t="s">
-        <v>27</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -712,55 +705,55 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>56</v>
       </c>
       <c r="C13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D13">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="C14" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D14">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="D15">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B16" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C16" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="D16">
         <v>0</v>
@@ -768,27 +761,27 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="B17" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="C17" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="D17">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="B18" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C18" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="D18">
         <v>1</v>
@@ -796,30 +789,16 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B19" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C19" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="D19">
         <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>58</v>
-      </c>
-      <c r="B20" t="s">
-        <v>59</v>
-      </c>
-      <c r="C20" t="s">
-        <v>60</v>
-      </c>
-      <c r="D20">
-        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>